<commit_message>
feat(go): add fuzzy-address customer code lookup for Satra
</commit_message>
<xml_diff>
--- a/GO/internal/processing/productdata/testdata/data.xlsx
+++ b/GO/internal/processing/productdata/testdata/data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Hệ thống</t>
   </si>
@@ -90,6 +90,18 @@
   </si>
   <si>
     <t>7654321</t>
+  </si>
+  <si>
+    <t>SATRA</t>
+  </si>
+  <si>
+    <t>666</t>
+  </si>
+  <si>
+    <t>MN_MT_TESTSTF</t>
+  </si>
+  <si>
+    <t>123 Nguyễn Huệ, Phường Bến Nghé, Quận 1, Tp.HCM, VNM</t>
   </si>
 </sst>
 </file>
@@ -446,6 +458,20 @@
         <v>13</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(go): guard blank column A in fuzzy-address customer lookup
Mirrors Python's "if col_A and ..." truthiness check
(laymakhachhang_satra, xulydonhang.py:278). Without it,
strings.Contains(x, "") is always true in Go, so a row with a blank
column A would wrongly pass the system filter for every query.

Adds a fixture row (blank column A, populated column D) and a
regression test proving such rows never match, for any system.
</commit_message>
<xml_diff>
--- a/GO/internal/processing/productdata/testdata/data.xlsx
+++ b/GO/internal/processing/productdata/testdata/data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Hệ thống</t>
   </si>
@@ -102,6 +102,18 @@
   </si>
   <si>
     <t>123 Nguyễn Huệ, Phường Bến Nghé, Quận 1, Tp.HCM, VNM</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>555</t>
+  </si>
+  <si>
+    <t>BLANK_A_TESTCODE</t>
+  </si>
+  <si>
+    <t>456 Le Loi, Phuong Ben Thanh, Quan 1, Tp.HCM, VNM</t>
   </si>
 </sst>
 </file>
@@ -472,6 +484,20 @@
         <v>28</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(go): dispatch RealProcessor to Winmart via processWinmartSegment
Adds winmart_processor.go (processWinmartSegment, winmartRegionInfo,
winmartOrderNumber), wires a new "Winmart" case into Process's per-page
dispatch switch, and extends the shared productdata test fixture with a
WINMART row. Reuses buildPromoBonusRow unmodified for per-item bonus
rows (confirmed structurally identical to Coop's index==0 case); the
invoice-level bonus row gets its own inline block since Winmart writes
only the first matched SKU to column Q, unlike the shared
buildInvoiceBonusRow's joined-list behavior. The zero-price "giao rời"
skip is a deliberate divergence from Python's real (buggy) absolute-row
check, scoped to only mark rows within the current order.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GO/internal/processing/productdata/testdata/data.xlsx
+++ b/GO/internal/processing/productdata/testdata/data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>Hệ thống</t>
   </si>
@@ -126,6 +126,18 @@
   </si>
   <si>
     <t>BigC Test Product B</t>
+  </si>
+  <si>
+    <t>WINMART</t>
+  </si>
+  <si>
+    <t>WM001</t>
+  </si>
+  <si>
+    <t>MN_MT_TESTWIN</t>
+  </si>
+  <si>
+    <t>789 Trần Hưng Đạo, Phường Cầu Kho, Quận 1, Tp.HCM, VNM</t>
   </si>
 </sst>
 </file>
@@ -510,6 +522,20 @@
         <v>32</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>